<commit_message>
Review sheet: an answer's date comes from the sheet, as a decision's does
The Questions tab had no Date column, so an answer was always dated the day
review apply ran. Rebuilding the example from a requirement gave a different
file every day, and its check failed from the day after it was committed. The
tab now has a Date column: the date written there, or today when it is empty,
and a date that isn't one is refused. The example's sheet carries its dates.
</commit_message>
<xml_diff>
--- a/examples/from-a-requirement/review/1-criteria.xlsx
+++ b/examples/from-a-requirement/review/1-criteria.xlsx
@@ -906,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -915,6 +915,7 @@
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -948,6 +949,11 @@
           <t>Answered by</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -980,6 +986,11 @@
           <t>product-owner</t>
         </is>
       </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1012,6 +1023,11 @@
           <t>product-owner</t>
         </is>
       </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1042,6 +1058,11 @@
       <c r="F4" s="4" t="inlineStr">
         <is>
           <t>product-owner</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>

</xml_diff>